<commit_message>
Bug-003-Current ITR- Previous Itr
</commit_message>
<xml_diff>
--- a/app/zen_rules/bank_Company_Organization_Eligibility_Matrix.xlsx
+++ b/app/zen_rules/bank_Company_Organization_Eligibility_Matrix.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="58">
   <si>
     <t>Bank Name</t>
   </si>
@@ -152,6 +152,9 @@
   </si>
   <si>
     <t>&gt;= 726</t>
+  </si>
+  <si>
+    <t>condition</t>
   </si>
   <si>
     <t>Current + Prev &gt;= 600000</t>
@@ -919,10 +922,10 @@
         <v>28</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="S5" s="1" t="s">
         <v>29</v>
@@ -948,13 +951,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>28</v>
@@ -978,7 +981,7 @@
         <v>29</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="L6" s="1" t="s">
         <v>31</v>
@@ -1025,10 +1028,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>27</v>
@@ -1102,10 +1105,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>27</v>
@@ -1179,10 +1182,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>27</v>

</xml_diff>